<commit_message>
feat: implement Paldea routes & generate regional XLSX files\n\n- Add `paldeaRoutes.js` and `paldeaMapCoordinates.js` to `config/` derived from raw user input.\n- Add Region 10 (Paldea) to `pokedexIndexes.js` (Gen 9 ids 906-1025).\n- Generated regional Excel data files (`.xlsx`) for Regions 6 through 10, populated with validation data, calculated rarity formatting, challenge/unlock associations, and traced base evolution obtainability for unplaced Pokemon.\n- Fixed issues where challenges in Kalos were incorrectly exported, causing blank sheets, and removed the "Legacy" tag placeholder as requested.
Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/7_Alola_Data.xlsx
+++ b/7_Alola_Data.xlsx
@@ -460,7 +460,7 @@
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H2" t="str">
         <v>Ok</v>
@@ -498,7 +498,7 @@
         <v/>
       </c>
       <c r="G3" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H3" t="str">
         <v>Ok</v>
@@ -536,7 +536,7 @@
         <v/>
       </c>
       <c r="G4" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H4" t="str">
         <v>Ok</v>
@@ -574,7 +574,7 @@
         <v/>
       </c>
       <c r="G5" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H5" t="str">
         <v>Ok</v>
@@ -612,7 +612,7 @@
         <v/>
       </c>
       <c r="G6" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H6" t="str">
         <v>Ok</v>
@@ -650,7 +650,7 @@
         <v/>
       </c>
       <c r="G7" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H7" t="str">
         <v>Ok</v>
@@ -688,7 +688,7 @@
         <v/>
       </c>
       <c r="G8" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H8" t="str">
         <v>Ok</v>
@@ -726,7 +726,7 @@
         <v/>
       </c>
       <c r="G9" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H9" t="str">
         <v>Ok</v>
@@ -764,7 +764,7 @@
         <v/>
       </c>
       <c r="G10" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H10" t="str">
         <v>Ok</v>
@@ -802,7 +802,7 @@
         <v/>
       </c>
       <c r="G11" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H11" t="str">
         <v>Ok</v>
@@ -840,7 +840,7 @@
         <v/>
       </c>
       <c r="G12" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H12" t="str">
         <v>Ok</v>
@@ -878,7 +878,7 @@
         <v/>
       </c>
       <c r="G13" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H13" t="str">
         <v>Ok</v>
@@ -916,7 +916,7 @@
         <v/>
       </c>
       <c r="G14" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H14" t="str">
         <v>Ok</v>
@@ -954,7 +954,7 @@
         <v/>
       </c>
       <c r="G15" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H15" t="str">
         <v>Ok</v>
@@ -992,7 +992,7 @@
         <v/>
       </c>
       <c r="G16" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H16" t="str">
         <v>Ok</v>
@@ -1030,7 +1030,7 @@
         <v/>
       </c>
       <c r="G17" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H17" t="str">
         <v>Ok</v>
@@ -1068,7 +1068,7 @@
         <v/>
       </c>
       <c r="G18" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H18" t="str">
         <v>Ok</v>
@@ -1106,7 +1106,7 @@
         <v/>
       </c>
       <c r="G19" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H19" t="str">
         <v>Ok</v>
@@ -1144,7 +1144,7 @@
         <v/>
       </c>
       <c r="G20" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H20" t="str">
         <v>Ok</v>
@@ -1182,7 +1182,7 @@
         <v/>
       </c>
       <c r="G21" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H21" t="str">
         <v>Ok</v>
@@ -1258,7 +1258,7 @@
         <v/>
       </c>
       <c r="G23" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H23" t="str">
         <v>Ok</v>
@@ -1296,7 +1296,7 @@
         <v/>
       </c>
       <c r="G24" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H24" t="str">
         <v>Ok</v>
@@ -1334,7 +1334,7 @@
         <v/>
       </c>
       <c r="G25" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H25" t="str">
         <v>Ok</v>
@@ -1372,7 +1372,7 @@
         <v/>
       </c>
       <c r="G26" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H26" t="str">
         <v>Ok</v>
@@ -1410,7 +1410,7 @@
         <v/>
       </c>
       <c r="G27" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H27" t="str">
         <v>Ok</v>
@@ -1448,7 +1448,7 @@
         <v/>
       </c>
       <c r="G28" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H28" t="str">
         <v>NONONO</v>
@@ -1486,7 +1486,7 @@
         <v/>
       </c>
       <c r="G29" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H29" t="str">
         <v>Ok</v>
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="G30" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H30" t="str">
         <v>Ok</v>
@@ -1562,7 +1562,7 @@
         <v/>
       </c>
       <c r="G31" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H31" t="str">
         <v>Ok</v>
@@ -1600,7 +1600,7 @@
         <v/>
       </c>
       <c r="G32" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H32" t="str">
         <v>Ok</v>
@@ -1638,7 +1638,7 @@
         <v/>
       </c>
       <c r="G33" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H33" t="str">
         <v>Ok</v>
@@ -1676,7 +1676,7 @@
         <v/>
       </c>
       <c r="G34" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H34" t="str">
         <v>Ok</v>
@@ -1714,7 +1714,7 @@
         <v/>
       </c>
       <c r="G35" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H35" t="str">
         <v>Ok</v>
@@ -1790,7 +1790,7 @@
         <v/>
       </c>
       <c r="G37" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H37" t="str">
         <v>Ok</v>
@@ -1828,7 +1828,7 @@
         <v/>
       </c>
       <c r="G38" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H38" t="str">
         <v>Ok</v>
@@ -1866,7 +1866,7 @@
         <v/>
       </c>
       <c r="G39" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H39" t="str">
         <v>Ok</v>
@@ -1904,7 +1904,7 @@
         <v/>
       </c>
       <c r="G40" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H40" t="str">
         <v>Ok</v>
@@ -1980,7 +1980,7 @@
         <v/>
       </c>
       <c r="G42" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H42" t="str">
         <v>Ok</v>
@@ -2018,7 +2018,7 @@
         <v/>
       </c>
       <c r="G43" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H43" t="str">
         <v>Ok</v>
@@ -2056,7 +2056,7 @@
         <v/>
       </c>
       <c r="G44" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H44" t="str">
         <v>Ok</v>
@@ -2094,7 +2094,7 @@
         <v/>
       </c>
       <c r="G45" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H45" t="str">
         <v>Ok</v>
@@ -2170,7 +2170,7 @@
         <v/>
       </c>
       <c r="G47" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H47" t="str">
         <v>Ok</v>
@@ -2208,7 +2208,7 @@
         <v/>
       </c>
       <c r="G48" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H48" t="str">
         <v>Ok</v>
@@ -2246,7 +2246,7 @@
         <v/>
       </c>
       <c r="G49" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H49" t="str">
         <v>Ok</v>
@@ -2322,7 +2322,7 @@
         <v/>
       </c>
       <c r="G51" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H51" t="str">
         <v>Ok</v>
@@ -2360,7 +2360,7 @@
         <v/>
       </c>
       <c r="G52" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H52" t="str">
         <v>Ok</v>
@@ -2398,7 +2398,7 @@
         <v/>
       </c>
       <c r="G53" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H53" t="str">
         <v>Ok</v>
@@ -2436,7 +2436,7 @@
         <v/>
       </c>
       <c r="G54" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H54" t="str">
         <v>Ok</v>
@@ -2474,7 +2474,7 @@
         <v/>
       </c>
       <c r="G55" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H55" t="str">
         <v>Ok</v>
@@ -2512,7 +2512,7 @@
         <v/>
       </c>
       <c r="G56" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H56" t="str">
         <v>Ok</v>
@@ -2550,7 +2550,7 @@
         <v/>
       </c>
       <c r="G57" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H57" t="str">
         <v>Ok</v>
@@ -2588,7 +2588,7 @@
         <v/>
       </c>
       <c r="G58" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H58" t="str">
         <v>Ok</v>
@@ -2626,7 +2626,7 @@
         <v/>
       </c>
       <c r="G59" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H59" t="str">
         <v>Ok</v>
@@ -2664,7 +2664,7 @@
         <v/>
       </c>
       <c r="G60" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H60" t="str">
         <v>Ok</v>
@@ -2702,7 +2702,7 @@
         <v/>
       </c>
       <c r="G61" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H61" t="str">
         <v>Ok</v>
@@ -2740,7 +2740,7 @@
         <v/>
       </c>
       <c r="G62" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H62" t="str">
         <v>Ok</v>
@@ -2778,7 +2778,7 @@
         <v/>
       </c>
       <c r="G63" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H63" t="str">
         <v>Ok</v>
@@ -2816,7 +2816,7 @@
         <v/>
       </c>
       <c r="G64" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H64" t="str">
         <v>Ok</v>
@@ -2854,7 +2854,7 @@
         <v/>
       </c>
       <c r="G65" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H65" t="str">
         <v>Ok</v>
@@ -2892,7 +2892,7 @@
         <v/>
       </c>
       <c r="G66" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H66" t="str">
         <v>Ok</v>
@@ -2930,7 +2930,7 @@
         <v/>
       </c>
       <c r="G67" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H67" t="str">
         <v>Ok</v>
@@ -2968,7 +2968,7 @@
         <v/>
       </c>
       <c r="G68" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H68" t="str">
         <v>Ok</v>
@@ -3006,7 +3006,7 @@
         <v/>
       </c>
       <c r="G69" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H69" t="str">
         <v>Ok</v>
@@ -3044,7 +3044,7 @@
         <v/>
       </c>
       <c r="G70" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H70" t="str">
         <v>Ok</v>
@@ -3082,7 +3082,7 @@
         <v/>
       </c>
       <c r="G71" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H71" t="str">
         <v>Ok</v>
@@ -3120,7 +3120,7 @@
         <v/>
       </c>
       <c r="G72" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H72" t="str">
         <v>Ok</v>
@@ -3158,7 +3158,7 @@
         <v/>
       </c>
       <c r="G73" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H73" t="str">
         <v>Ok</v>
@@ -3196,7 +3196,7 @@
         <v/>
       </c>
       <c r="G74" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H74" t="str">
         <v>Ok</v>
@@ -3234,7 +3234,7 @@
         <v/>
       </c>
       <c r="G75" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H75" t="str">
         <v>Ok</v>
@@ -3272,7 +3272,7 @@
         <v/>
       </c>
       <c r="G76" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H76" t="str">
         <v>Ok</v>
@@ -3310,7 +3310,7 @@
         <v/>
       </c>
       <c r="G77" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H77" t="str">
         <v>Ok</v>
@@ -3348,7 +3348,7 @@
         <v/>
       </c>
       <c r="G78" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H78" t="str">
         <v>Ok</v>
@@ -3424,7 +3424,7 @@
         <v/>
       </c>
       <c r="G80" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H80" t="str">
         <v>Ok</v>
@@ -3462,7 +3462,7 @@
         <v/>
       </c>
       <c r="G81" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H81" t="str">
         <v>Ok</v>
@@ -3500,7 +3500,7 @@
         <v/>
       </c>
       <c r="G82" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H82" t="str">
         <v>Ok</v>
@@ -3538,7 +3538,7 @@
         <v/>
       </c>
       <c r="G83" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H83" t="str">
         <v>Ok</v>
@@ -3576,7 +3576,7 @@
         <v/>
       </c>
       <c r="G84" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H84" t="str">
         <v>Ok</v>
@@ -3614,7 +3614,7 @@
         <v/>
       </c>
       <c r="G85" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H85" t="str">
         <v>Ok</v>
@@ -3652,7 +3652,7 @@
         <v/>
       </c>
       <c r="G86" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H86" t="str">
         <v>Ok</v>
@@ -3690,7 +3690,7 @@
         <v/>
       </c>
       <c r="G87" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H87" t="str">
         <v>Ok</v>
@@ -3728,7 +3728,7 @@
         <v/>
       </c>
       <c r="G88" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H88" t="str">
         <v>Ok</v>
@@ -3766,7 +3766,7 @@
         <v/>
       </c>
       <c r="G89" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H89" t="str">
         <v>Ok</v>
@@ -3804,7 +3804,7 @@
         <v/>
       </c>
       <c r="G90" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H90" t="str">
         <v>Ok</v>
@@ -3842,7 +3842,7 @@
         <v/>
       </c>
       <c r="G91" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H91" t="str">
         <v>Ok</v>
@@ -3918,7 +3918,7 @@
         <v/>
       </c>
       <c r="G93" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H93" t="str">
         <v>Ok</v>
@@ -3956,7 +3956,7 @@
         <v/>
       </c>
       <c r="G94" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H94" t="str">
         <v>Ok</v>
@@ -3994,7 +3994,7 @@
         <v/>
       </c>
       <c r="G95" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H95" t="str">
         <v>Ok</v>
@@ -4032,7 +4032,7 @@
         <v/>
       </c>
       <c r="G96" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H96" t="str">
         <v>Ok</v>
@@ -4070,7 +4070,7 @@
         <v/>
       </c>
       <c r="G97" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H97" t="str">
         <v>Ok</v>
@@ -4108,7 +4108,7 @@
         <v/>
       </c>
       <c r="G98" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H98" t="str">
         <v>Ok</v>
@@ -4146,7 +4146,7 @@
         <v/>
       </c>
       <c r="G99" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H99" t="str">
         <v>Ok</v>
@@ -4184,7 +4184,7 @@
         <v/>
       </c>
       <c r="G100" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H100" t="str">
         <v>Ok</v>
@@ -4222,7 +4222,7 @@
         <v/>
       </c>
       <c r="G101" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H101" t="str">
         <v>Ok</v>
@@ -4298,7 +4298,7 @@
         <v/>
       </c>
       <c r="G103" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H103" t="str">
         <v>Ok</v>
@@ -4336,7 +4336,7 @@
         <v/>
       </c>
       <c r="G104" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H104" t="str">
         <v>Ok</v>
@@ -4374,7 +4374,7 @@
         <v/>
       </c>
       <c r="G105" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H105" t="str">
         <v>Ok</v>
@@ -4412,7 +4412,7 @@
         <v/>
       </c>
       <c r="G106" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H106" t="str">
         <v>Ok</v>
@@ -4450,7 +4450,7 @@
         <v/>
       </c>
       <c r="G107" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H107" t="str">
         <v>Ok</v>
@@ -4488,7 +4488,7 @@
         <v/>
       </c>
       <c r="G108" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H108" t="str">
         <v>Ok</v>
@@ -4526,7 +4526,7 @@
         <v/>
       </c>
       <c r="G109" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H109" t="str">
         <v>Ok</v>
@@ -4564,7 +4564,7 @@
         <v/>
       </c>
       <c r="G110" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H110" t="str">
         <v>Ok</v>
@@ -4602,7 +4602,7 @@
         <v/>
       </c>
       <c r="G111" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H111" t="str">
         <v>Ok</v>
@@ -4640,7 +4640,7 @@
         <v/>
       </c>
       <c r="G112" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H112" t="str">
         <v>Ok</v>
@@ -4678,7 +4678,7 @@
         <v/>
       </c>
       <c r="G113" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H113" t="str">
         <v>Ok</v>
@@ -4716,7 +4716,7 @@
         <v/>
       </c>
       <c r="G114" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H114" t="str">
         <v>Ok</v>
@@ -4754,7 +4754,7 @@
         <v/>
       </c>
       <c r="G115" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H115" t="str">
         <v>Ok</v>
@@ -4792,7 +4792,7 @@
         <v/>
       </c>
       <c r="G116" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H116" t="str">
         <v>Ok</v>
@@ -4830,7 +4830,7 @@
         <v/>
       </c>
       <c r="G117" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H117" t="str">
         <v>Ok</v>
@@ -4868,7 +4868,7 @@
         <v/>
       </c>
       <c r="G118" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H118" t="str">
         <v>Ok</v>
@@ -4982,7 +4982,7 @@
         <v/>
       </c>
       <c r="G121" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H121" t="str">
         <v>Ok</v>
@@ -5020,7 +5020,7 @@
         <v/>
       </c>
       <c r="G122" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H122" t="str">
         <v>Ok</v>
@@ -5058,7 +5058,7 @@
         <v/>
       </c>
       <c r="G123" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H123" t="str">
         <v>Ok</v>
@@ -5096,7 +5096,7 @@
         <v/>
       </c>
       <c r="G124" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H124" t="str">
         <v>Ok</v>
@@ -5134,7 +5134,7 @@
         <v/>
       </c>
       <c r="G125" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H125" t="str">
         <v>Ok</v>
@@ -5172,7 +5172,7 @@
         <v/>
       </c>
       <c r="G126" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H126" t="str">
         <v>Ok</v>
@@ -5210,7 +5210,7 @@
         <v/>
       </c>
       <c r="G127" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H127" t="str">
         <v>Ok</v>
@@ -5248,7 +5248,7 @@
         <v/>
       </c>
       <c r="G128" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H128" t="str">
         <v>Ok</v>
@@ -5286,7 +5286,7 @@
         <v/>
       </c>
       <c r="G129" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H129" t="str">
         <v>Ok</v>
@@ -5324,7 +5324,7 @@
         <v/>
       </c>
       <c r="G130" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H130" t="str">
         <v>Ok</v>
@@ -5362,7 +5362,7 @@
         <v/>
       </c>
       <c r="G131" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H131" t="str">
         <v>Ok</v>
@@ -5400,7 +5400,7 @@
         <v/>
       </c>
       <c r="G132" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H132" t="str">
         <v>Ok</v>
@@ -5438,7 +5438,7 @@
         <v/>
       </c>
       <c r="G133" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H133" t="str">
         <v>Ok</v>
@@ -5476,7 +5476,7 @@
         <v/>
       </c>
       <c r="G134" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H134" t="str">
         <v>Ok</v>
@@ -5514,7 +5514,7 @@
         <v/>
       </c>
       <c r="G135" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H135" t="str">
         <v>Ok</v>
@@ -5552,7 +5552,7 @@
         <v/>
       </c>
       <c r="G136" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H136" t="str">
         <v>Ok</v>
@@ -5590,7 +5590,7 @@
         <v/>
       </c>
       <c r="G137" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H137" t="str">
         <v>Ok</v>
@@ -5628,7 +5628,7 @@
         <v/>
       </c>
       <c r="G138" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H138" t="str">
         <v>Ok</v>
@@ -5666,7 +5666,7 @@
         <v/>
       </c>
       <c r="G139" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H139" t="str">
         <v>Ok</v>
@@ -5704,7 +5704,7 @@
         <v/>
       </c>
       <c r="G140" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H140" t="str">
         <v>Ok</v>
@@ -5742,7 +5742,7 @@
         <v/>
       </c>
       <c r="G141" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H141" t="str">
         <v>Ok</v>
@@ -5780,7 +5780,7 @@
         <v/>
       </c>
       <c r="G142" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H142" t="str">
         <v>Ok</v>
@@ -5818,7 +5818,7 @@
         <v/>
       </c>
       <c r="G143" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H143" t="str">
         <v>Ok</v>
@@ -5970,7 +5970,7 @@
         <v/>
       </c>
       <c r="G147" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H147" t="str">
         <v>Ok</v>
@@ -6008,7 +6008,7 @@
         <v/>
       </c>
       <c r="G148" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H148" t="str">
         <v>Ok</v>
@@ -6046,7 +6046,7 @@
         <v/>
       </c>
       <c r="G149" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H149" t="str">
         <v>Ok</v>
@@ -6084,7 +6084,7 @@
         <v/>
       </c>
       <c r="G150" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H150" t="str">
         <v>Ok</v>
@@ -6502,7 +6502,7 @@
         <v/>
       </c>
       <c r="G161" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H161" t="str">
         <v>Ok</v>
@@ -6540,7 +6540,7 @@
         <v/>
       </c>
       <c r="G162" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H162" t="str">
         <v>Ok</v>
@@ -6578,7 +6578,7 @@
         <v/>
       </c>
       <c r="G163" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H163" t="str">
         <v>Ok</v>
@@ -6616,7 +6616,7 @@
         <v/>
       </c>
       <c r="G164" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H164" t="str">
         <v>NONONO</v>
@@ -6654,7 +6654,7 @@
         <v/>
       </c>
       <c r="G165" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H165" t="str">
         <v>Ok</v>
@@ -6692,7 +6692,7 @@
         <v/>
       </c>
       <c r="G166" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H166" t="str">
         <v>NONONO</v>
@@ -6730,7 +6730,7 @@
         <v/>
       </c>
       <c r="G167" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H167" t="str">
         <v>NONONO</v>
@@ -6768,7 +6768,7 @@
         <v/>
       </c>
       <c r="G168" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H168" t="str">
         <v>NONONO</v>
@@ -6806,7 +6806,7 @@
         <v/>
       </c>
       <c r="G169" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H169" t="str">
         <v>Ok</v>
@@ -6844,7 +6844,7 @@
         <v/>
       </c>
       <c r="G170" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H170" t="str">
         <v>NONONO</v>
@@ -6882,7 +6882,7 @@
         <v/>
       </c>
       <c r="G171" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H171" t="str">
         <v>Ok</v>
@@ -6920,7 +6920,7 @@
         <v/>
       </c>
       <c r="G172" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H172" t="str">
         <v>NONONO</v>
@@ -6958,7 +6958,7 @@
         <v/>
       </c>
       <c r="G173" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H173" t="str">
         <v>Ok</v>
@@ -6996,7 +6996,7 @@
         <v/>
       </c>
       <c r="G174" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H174" t="str">
         <v>Ok</v>
@@ -7034,7 +7034,7 @@
         <v/>
       </c>
       <c r="G175" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H175" t="str">
         <v>Ok</v>
@@ -7072,7 +7072,7 @@
         <v/>
       </c>
       <c r="G176" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H176" t="str">
         <v>Ok</v>
@@ -7110,7 +7110,7 @@
         <v/>
       </c>
       <c r="G177" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H177" t="str">
         <v>Ok</v>
@@ -7148,7 +7148,7 @@
         <v/>
       </c>
       <c r="G178" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H178" t="str">
         <v>Ok</v>
@@ -7186,7 +7186,7 @@
         <v/>
       </c>
       <c r="G179" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H179" t="str">
         <v>Ok</v>
@@ -7224,7 +7224,7 @@
         <v/>
       </c>
       <c r="G180" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H180" t="str">
         <v>Ok</v>
@@ -7262,7 +7262,7 @@
         <v/>
       </c>
       <c r="G181" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H181" t="str">
         <v>Ok</v>
@@ -7300,7 +7300,7 @@
         <v/>
       </c>
       <c r="G182" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H182" t="str">
         <v>NONONO</v>
@@ -7338,7 +7338,7 @@
         <v/>
       </c>
       <c r="G183" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H183" t="str">
         <v>Ok</v>
@@ -7376,7 +7376,7 @@
         <v/>
       </c>
       <c r="G184" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H184" t="str">
         <v>Ok</v>
@@ -7414,7 +7414,7 @@
         <v/>
       </c>
       <c r="G185" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H185" t="str">
         <v>Ok</v>
@@ -7452,7 +7452,7 @@
         <v/>
       </c>
       <c r="G186" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H186" t="str">
         <v>Ok</v>
@@ -7490,7 +7490,7 @@
         <v/>
       </c>
       <c r="G187" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H187" t="str">
         <v>Ok</v>
@@ -7528,7 +7528,7 @@
         <v/>
       </c>
       <c r="G188" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H188" t="str">
         <v>Ok</v>
@@ -7566,7 +7566,7 @@
         <v/>
       </c>
       <c r="G189" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H189" t="str">
         <v>Ok</v>
@@ -7604,7 +7604,7 @@
         <v/>
       </c>
       <c r="G190" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H190" t="str">
         <v>NONONO</v>
@@ -7642,7 +7642,7 @@
         <v/>
       </c>
       <c r="G191" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H191" t="str">
         <v>NONONO</v>
@@ -7680,7 +7680,7 @@
         <v/>
       </c>
       <c r="G192" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H192" t="str">
         <v>NONONO</v>
@@ -7718,7 +7718,7 @@
         <v/>
       </c>
       <c r="G193" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H193" t="str">
         <v>Ok</v>
@@ -7756,7 +7756,7 @@
         <v/>
       </c>
       <c r="G194" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H194" t="str">
         <v>NONONO</v>
@@ -7794,7 +7794,7 @@
         <v/>
       </c>
       <c r="G195" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H195" t="str">
         <v>NONONO</v>
@@ -7832,7 +7832,7 @@
         <v/>
       </c>
       <c r="G196" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H196" t="str">
         <v>NONONO</v>
@@ -7870,7 +7870,7 @@
         <v/>
       </c>
       <c r="G197" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H197" t="str">
         <v>NONONO</v>
@@ -7908,7 +7908,7 @@
         <v/>
       </c>
       <c r="G198" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H198" t="str">
         <v>NONONO</v>
@@ -7946,7 +7946,7 @@
         <v/>
       </c>
       <c r="G199" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H199" t="str">
         <v>NONONO</v>
@@ -7984,7 +7984,7 @@
         <v/>
       </c>
       <c r="G200" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H200" t="str">
         <v>NONONO</v>
@@ -8022,7 +8022,7 @@
         <v/>
       </c>
       <c r="G201" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H201" t="str">
         <v>Ok</v>
@@ -8060,7 +8060,7 @@
         <v/>
       </c>
       <c r="G202" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H202" t="str">
         <v>Ok</v>
@@ -8098,7 +8098,7 @@
         <v/>
       </c>
       <c r="G203" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H203" t="str">
         <v>Ok</v>
@@ -8136,7 +8136,7 @@
         <v/>
       </c>
       <c r="G204" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H204" t="str">
         <v>Ok</v>
@@ -8174,7 +8174,7 @@
         <v/>
       </c>
       <c r="G205" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H205" t="str">
         <v>Ok</v>
@@ -8212,7 +8212,7 @@
         <v/>
       </c>
       <c r="G206" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H206" t="str">
         <v>Ok</v>
@@ -8250,7 +8250,7 @@
         <v/>
       </c>
       <c r="G207" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H207" t="str">
         <v>NONONO</v>
@@ -8288,7 +8288,7 @@
         <v/>
       </c>
       <c r="G208" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H208" t="str">
         <v>Ok</v>
@@ -8326,7 +8326,7 @@
         <v/>
       </c>
       <c r="G209" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H209" t="str">
         <v>Ok</v>
@@ -8364,7 +8364,7 @@
         <v/>
       </c>
       <c r="G210" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H210" t="str">
         <v>Ok</v>
@@ -8402,7 +8402,7 @@
         <v/>
       </c>
       <c r="G211" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H211" t="str">
         <v>Ok</v>
@@ -8440,7 +8440,7 @@
         <v/>
       </c>
       <c r="G212" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H212" t="str">
         <v>Ok</v>
@@ -8478,7 +8478,7 @@
         <v/>
       </c>
       <c r="G213" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H213" t="str">
         <v>Ok</v>
@@ -8516,7 +8516,7 @@
         <v/>
       </c>
       <c r="G214" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H214" t="str">
         <v>Ok</v>
@@ -8554,7 +8554,7 @@
         <v/>
       </c>
       <c r="G215" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H215" t="str">
         <v>Ok</v>
@@ -8592,7 +8592,7 @@
         <v/>
       </c>
       <c r="G216" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H216" t="str">
         <v>Ok</v>
@@ -8630,7 +8630,7 @@
         <v/>
       </c>
       <c r="G217" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H217" t="str">
         <v>Ok</v>
@@ -8668,7 +8668,7 @@
         <v/>
       </c>
       <c r="G218" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H218" t="str">
         <v>Ok</v>
@@ -8706,7 +8706,7 @@
         <v/>
       </c>
       <c r="G219" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H219" t="str">
         <v>Ok</v>
@@ -8744,7 +8744,7 @@
         <v/>
       </c>
       <c r="G220" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H220" t="str">
         <v>NONONO</v>
@@ -8782,7 +8782,7 @@
         <v/>
       </c>
       <c r="G221" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H221" t="str">
         <v>Ok</v>
@@ -8820,7 +8820,7 @@
         <v/>
       </c>
       <c r="G222" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H222" t="str">
         <v>Ok</v>
@@ -8858,7 +8858,7 @@
         <v/>
       </c>
       <c r="G223" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H223" t="str">
         <v>NONONO</v>
@@ -8896,7 +8896,7 @@
         <v/>
       </c>
       <c r="G224" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H224" t="str">
         <v>Ok</v>
@@ -8934,7 +8934,7 @@
         <v/>
       </c>
       <c r="G225" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H225" t="str">
         <v>NONONO</v>
@@ -8972,7 +8972,7 @@
         <v/>
       </c>
       <c r="G226" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H226" t="str">
         <v>Ok</v>
@@ -9010,7 +9010,7 @@
         <v/>
       </c>
       <c r="G227" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H227" t="str">
         <v>Ok</v>
@@ -9048,7 +9048,7 @@
         <v/>
       </c>
       <c r="G228" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H228" t="str">
         <v>Ok</v>
@@ -9086,7 +9086,7 @@
         <v/>
       </c>
       <c r="G229" t="str">
-        <v>Legacy</v>
+        <v/>
       </c>
       <c r="H229" t="str">
         <v>Ok</v>

</xml_diff>